<commit_message>
ignoring the hype / live keywords in actual and expected data because of its dynamic nature while asseertions
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV Ophef YouTube Premium YouTube Kids Aangeegeskiedenis</t>
+          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV YouTube Premium YouTube Kids Aangeegeskiedenis</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV Hayp YouTube Premium YouTube Kids Xəbər tarixçəsi</t>
+          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV YouTube Premium YouTube Kids Xəbər tarixçəsi</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV Beri hype YouTube Premium YouTube Kids Histori laporan</t>
+          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV YouTube Premium YouTube Kids Histori laporan</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV Poticanje interesovanja YouTube Premium YouTube Kids Historija prijava</t>
+          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV YouTube Premium YouTube Kids Historija prijava</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió Hype YouTube Premium YouTube Kids Historial d'informes</t>
+          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió YouTube Premium YouTube Kids Historial d'informes</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv Hype YouTube Premium YouTube Kids Rapporteringshistorik</t>
+          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv YouTube Premium YouTube Kids Rapporteringshistorik</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows Hype YouTube Premium YouTube Kids Meldeverlauf</t>
+          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows YouTube Premium YouTube Kids Meldeverlauf</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad Haipimine YouTube Premium YouTube Kids Teavituste ajalugu</t>
+          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad YouTube Premium YouTube Kids Teavituste ajalugu</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV YouTube Premium YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV YouTube Premium YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV YouTube Premium YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series Hype YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series YouTube Premium YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV YouTube Premium YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV YouTube Premium YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak Ikusmin-adierazpenak YouTube Premium YouTube Kids Salaketa-historia</t>
+          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak YouTube Premium YouTube Kids Salaketa-historia</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV Boost YouTube Premium YouTube Kids Signalements</t>
+          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV YouTube Premium YouTube Kids Signalements</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision Applaudissement YouTube Premium YouTube Kids Historique des rapports</t>
+          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision YouTube Premium YouTube Kids Historique des rapports</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija Razglašavanje YouTube Premium YouTube Kids Povijest prijava</t>
+          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija YouTube Premium YouTube Kids Povijest prijava</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni Upphefja YouTube Premium YouTube Kids Tilkynningaferill</t>
+          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni YouTube Premium YouTube Kids Tilkynningaferill</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV Hype YouTube Premium YouTube Kids Segnalazioni</t>
+          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV YouTube Premium YouTube Kids Segnalazioni</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides Popularizēšana YouTube Premium YouTube Kids Ziņošanas vēsture</t>
+          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides YouTube Premium YouTube Kids Ziņošanas vēsture</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV Pagyrimai YouTube Premium YouTube Kids Pranešimų istorija</t>
+          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV YouTube Premium YouTube Kids Pranešimų istorija</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé Hájpolás YouTube Premium YouTube Kids Bejelentési előzmények</t>
+          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé YouTube Premium YouTube Kids Bejelentési előzmények</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv Hype YouTube Premium YouTube Kids Rapportagegeschiedenis</t>
+          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv YouTube Premium YouTube Kids Rapportagegeschiedenis</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV Podbijanie YouTube Premium YouTube Kids Historia zgłoszeń</t>
+          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV YouTube Premium YouTube Kids Historia zgłoszeń</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV Hype YouTube Premium YouTube Kids Histórico de denúncias</t>
+          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV YouTube Premium YouTube Kids Histórico de denúncias</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV Hype YouTube Premium YouTube Kids Histórico de denúncias</t>
+          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV YouTube Premium YouTube Kids Histórico de denúncias</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni Popullarizo YouTube Premium YouTube Kids Historiku i raportimeve</t>
+          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni YouTube Premium YouTube Kids Historiku i raportimeve</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV Izražanje navdušenja YouTube Premium YouTube Kids Zgodovina poročil</t>
+          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV YouTube Premium YouTube Kids Zgodovina poročil</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV Hypetys YouTube Premium YouTube Kids Ilmoitushistoria</t>
+          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV YouTube Premium YouTube Kids Ilmoitushistoria</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv Hajp YouTube Premium YouTube Kids Rapporthistorik</t>
+          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv YouTube Premium YouTube Kids Rapporthistorik</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình Khuấy động YouTube Premium YouTube Kids Nhật ký báo cáo</t>
+          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình YouTube Premium YouTube Kids Nhật ký báo cáo</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV Hype YouTube Premium YouTube Kids İçerik bildirme geçmişi</t>
+          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV YouTube Premium YouTube Kids İçerik bildirme geçmişi</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы Галасаванне YouTube Premium YouTube Kids Гісторыя скаргаў</t>
+          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы YouTube Premium YouTube Kids Гісторыя скаргаў</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания Хайп YouTube Premium YouTube Kids Подадени сигнали</t>
+          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания YouTube Premium YouTube Kids Подадени сигнали</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы Хайп YouTube Premium YouTube Детям Жалобы</t>
+          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы YouTube Premium YouTube Детям Жалобы</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали Голосування YouTube Premium YouTube Kids Історія скарг</t>
+          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали YouTube Premium YouTube Kids Історія скарг</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές Hype YouTube Premium YouTube Kids Ιστορικό αναφορών</t>
+          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές YouTube Premium YouTube Kids Ιστορικό αναφορών</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ Հայփել YouTube Premium YouTube Kids Բողոքների պատմություն</t>
+          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ YouTube Premium YouTube Kids Բողոքների պատմություն</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה הייפ YouTube Premium YouTube Kids היסטוריית הדיווחים</t>
+          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה YouTube Premium YouTube Kids היסטוריית הדיווחים</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية التشجيع YouTube Premium YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
+          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية YouTube Premium YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون هیجان‌افزایی YouTube Premium YouTube Kids سابقه گزارش</t>
+          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون YouTube Premium YouTube Kids سابقه گزارش</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो हाइप YouTube Premium YouTube Kids शिकायतों का डेटा</t>
+          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो YouTube Premium YouTube Kids शिकायतों का डेटा</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি হাইপ YouTube Premium YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
+          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি YouTube Premium YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ ਹਾਈਪ ਕਰੋ YouTube Premium YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
+          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ YouTube Premium YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી હાઇપ YouTube Premium YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
+          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી YouTube Premium YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் ஹைப் YouTube Premium YouTube Kids புகார் வரலாறு</t>
+          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் YouTube Premium YouTube Kids புகார் வரலாறு</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ హైప్ YouTube Premium YouTube Kids రిపోర్టుల హిస్టరీ</t>
+          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ YouTube Premium YouTube Kids రిపోర్టుల హిస్టరీ</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 粉丝热推 YouTube Premium YouTube Kids 举报记录</t>
+          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 YouTube Premium YouTube Kids 举报记录</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 粉絲熱推 YouTube Premium YouTube Kids 檢舉記錄</t>
+          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 YouTube Premium YouTube Kids 檢舉記錄</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 粉絲推介 YouTube Premium YouTube Kids 舉報記錄</t>
+          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 YouTube Premium YouTube Kids 舉報記錄</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 ハイプ YouTube Premium YouTube Kids 報告履歴</t>
+          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 YouTube Premium YouTube Kids 報告履歴</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV 하이프 YouTube Premium YouTube Kids 신고 기록</t>
+          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV YouTube Premium YouTube Kids 신고 기록</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
checking the native live / hype word and smart checking it in assertions
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV YouTube Premium YouTube Kids Aangeegeskiedenis</t>
+          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV Ophef YouTube Premium YouTube Kids Aangeegeskiedenis</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV YouTube Premium YouTube Kids Xəbər tarixçəsi</t>
+          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV Hayp YouTube Premium YouTube Kids Xəbər tarixçəsi</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV YouTube Premium YouTube Kids Histori laporan</t>
+          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV Beri hype YouTube Premium YouTube Kids Histori laporan</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV YouTube Premium YouTube Kids Historija prijava</t>
+          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV Poticanje interesovanja YouTube Premium YouTube Kids Historija prijava</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió YouTube Premium YouTube Kids Historial d'informes</t>
+          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió Hype YouTube Premium YouTube Kids Historial d'informes</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv YouTube Premium YouTube Kids Rapporteringshistorik</t>
+          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv Hype YouTube Premium YouTube Kids Rapporteringshistorik</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows YouTube Premium YouTube Kids Meldeverlauf</t>
+          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows Hype YouTube Premium YouTube Kids Meldeverlauf</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad YouTube Premium YouTube Kids Teavituste ajalugu</t>
+          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad Haipimine YouTube Premium YouTube Kids Teavituste ajalugu</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series Hype YouTube Premium YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype YouTube Premium YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype YouTube Premium YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak YouTube Premium YouTube Kids Salaketa-historia</t>
+          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak Ikusmin-adierazpenak YouTube Premium YouTube Kids Salaketa-historia</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV YouTube Premium YouTube Kids Signalements</t>
+          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV Boost YouTube Premium YouTube Kids Signalements</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision YouTube Premium YouTube Kids Historique des rapports</t>
+          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision Applaudissement YouTube Premium YouTube Kids Historique des rapports</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija YouTube Premium YouTube Kids Povijest prijava</t>
+          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija Razglašavanje YouTube Premium YouTube Kids Povijest prijava</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni YouTube Premium YouTube Kids Tilkynningaferill</t>
+          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni Upphefja YouTube Premium YouTube Kids Tilkynningaferill</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV YouTube Premium YouTube Kids Segnalazioni</t>
+          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV Hype YouTube Premium YouTube Kids Segnalazioni</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides YouTube Premium YouTube Kids Ziņošanas vēsture</t>
+          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides Popularizēšana YouTube Premium YouTube Kids Ziņošanas vēsture</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV YouTube Premium YouTube Kids Pranešimų istorija</t>
+          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV Pagyrimai YouTube Premium YouTube Kids Pranešimų istorija</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé YouTube Premium YouTube Kids Bejelentési előzmények</t>
+          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé Hájpolás YouTube Premium YouTube Kids Bejelentési előzmények</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv YouTube Premium YouTube Kids Rapportagegeschiedenis</t>
+          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv Hype YouTube Premium YouTube Kids Rapportagegeschiedenis</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV YouTube Premium YouTube Kids Historia zgłoszeń</t>
+          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV Podbijanie YouTube Premium YouTube Kids Historia zgłoszeń</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV YouTube Premium YouTube Kids Histórico de denúncias</t>
+          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV Hype YouTube Premium YouTube Kids Histórico de denúncias</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV YouTube Premium YouTube Kids Histórico de denúncias</t>
+          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV Hype YouTube Premium YouTube Kids Histórico de denúncias</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni YouTube Premium YouTube Kids Historiku i raportimeve</t>
+          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni Popullarizo YouTube Premium YouTube Kids Historiku i raportimeve</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV YouTube Premium YouTube Kids Zgodovina poročil</t>
+          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV Izražanje navdušenja YouTube Premium YouTube Kids Zgodovina poročil</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV YouTube Premium YouTube Kids Ilmoitushistoria</t>
+          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV Hypetys YouTube Premium YouTube Kids Ilmoitushistoria</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv YouTube Premium YouTube Kids Rapporthistorik</t>
+          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv Hajp YouTube Premium YouTube Kids Rapporthistorik</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình YouTube Premium YouTube Kids Nhật ký báo cáo</t>
+          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình Khuấy động YouTube Premium YouTube Kids Nhật ký báo cáo</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV YouTube Premium YouTube Kids İçerik bildirme geçmişi</t>
+          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV Hype YouTube Premium YouTube Kids İçerik bildirme geçmişi</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы YouTube Premium YouTube Kids Гісторыя скаргаў</t>
+          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы Галасаванне YouTube Premium YouTube Kids Гісторыя скаргаў</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания YouTube Premium YouTube Kids Подадени сигнали</t>
+          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания Хайп YouTube Premium YouTube Kids Подадени сигнали</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы YouTube Premium YouTube Детям Жалобы</t>
+          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы Хайп YouTube Premium YouTube Детям Жалобы</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали YouTube Premium YouTube Kids Історія скарг</t>
+          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали Голосування YouTube Premium YouTube Kids Історія скарг</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές YouTube Premium YouTube Kids Ιστορικό αναφορών</t>
+          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές Hype YouTube Premium YouTube Kids Ιστορικό αναφορών</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ YouTube Premium YouTube Kids Բողոքների պատմություն</t>
+          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ Հայփել YouTube Premium YouTube Kids Բողոքների պատմություն</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה YouTube Premium YouTube Kids היסטוריית הדיווחים</t>
+          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה הייפ YouTube Premium YouTube Kids היסטוריית הדיווחים</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية YouTube Premium YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
+          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية التشجيع YouTube Premium YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون YouTube Premium YouTube Kids سابقه گزارش</t>
+          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون هیجان‌افزایی YouTube Premium YouTube Kids سابقه گزارش</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो YouTube Premium YouTube Kids शिकायतों का डेटा</t>
+          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो हाइप YouTube Premium YouTube Kids शिकायतों का डेटा</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি YouTube Premium YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
+          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি হাইপ YouTube Premium YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ YouTube Premium YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
+          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ ਹਾਈਪ ਕਰੋ YouTube Premium YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી YouTube Premium YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
+          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી હાઇપ YouTube Premium YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் YouTube Premium YouTube Kids புகார் வரலாறு</t>
+          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் ஹைப் YouTube Premium YouTube Kids புகார் வரலாறு</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ YouTube Premium YouTube Kids రిపోర్టుల హిస్టరీ</t>
+          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ హైప్ YouTube Premium YouTube Kids రిపోర్టుల హిస్టరీ</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 YouTube Premium YouTube Kids 举报记录</t>
+          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 粉丝热推 YouTube Premium YouTube Kids 举报记录</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 YouTube Premium YouTube Kids 檢舉記錄</t>
+          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 粉絲熱推 YouTube Premium YouTube Kids 檢舉記錄</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 YouTube Premium YouTube Kids 舉報記錄</t>
+          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 粉絲推介 YouTube Premium YouTube Kids 舉報記錄</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 YouTube Premium YouTube Kids 報告履歴</t>
+          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 ハイプ YouTube Premium YouTube Kids 報告履歴</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV YouTube Premium YouTube Kids 신고 기록</t>
+          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV 하이프 YouTube Premium YouTube Kids 신고 기록</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updating the side menu expected data with update yt changes
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV Ophef YouTube Premium YouTube Kids Aangeegeskiedenis</t>
+          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV Ophef Probeer Premium vir $0 YouTube Kids Aangeegeskiedenis</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV Hayp YouTube Premium YouTube Kids Xəbər tarixçəsi</t>
+          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV Hayp 0$-a Premium sınayın YouTube Kids Xəbər tarixçəsi</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV Beri hype YouTube Premium YouTube Kids Histori laporan</t>
+          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV Beri hype Coba Premium $0 YouTube Kids Histori laporan</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV Poticanje interesovanja YouTube Premium YouTube Kids Historija prijava</t>
+          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV Poticanje interesovanja Isprobajte Premium za 0 USD YouTube Kids Historija prijava</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió Hype YouTube Premium YouTube Kids Historial d'informes</t>
+          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió Hype Prova Premium per 0 € YouTube Kids Historial d'informes</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv Hype YouTube Premium YouTube Kids Rapporteringshistorik</t>
+          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv Hype Premium for 0 USD YouTube Kids Rapporteringshistorik</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows Hype YouTube Premium YouTube Kids Meldeverlauf</t>
+          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows Hype Premium kostenlos ausprobieren YouTube Kids Meldeverlauf</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad Haipimine YouTube Premium YouTube Kids Teavituste ajalugu</t>
+          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad Haipimine Premium 0 dollariga YouTube Kids Teavituste ajalugu</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype Try Premium for $0 YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype Try Premium for $0 YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype YouTube Premium YouTube Kids Report history</t>
+          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype Try Premium for $0 YouTube Kids Report history</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series Hype YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series Hype Probar Premium sin coste YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype Premium por USD 0 YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype YouTube Premium YouTube Kids Historial de denuncias</t>
+          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype Premium por USD 0 YouTube Kids Historial de denuncias</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak Ikusmin-adierazpenak YouTube Premium YouTube Kids Salaketa-historia</t>
+          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak Ikusmin-adierazpenak Probatu Premium 0 dolarrean YouTube Kids Salaketa-historia</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV Boost YouTube Premium YouTube Kids Signalements</t>
+          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV Boost Essayez Premium pour 0 $ YouTube Kids Signalements</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision Applaudissement YouTube Premium YouTube Kids Historique des rapports</t>
+          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision Applaudissement Essayez Premium pour 0 USD YouTube Kids Historique des rapports</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija Razglašavanje YouTube Premium YouTube Kids Povijest prijava</t>
+          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija Razglašavanje Isprobajte Premium za 0 USD YouTube Kids Povijest prijava</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni Upphefja YouTube Premium YouTube Kids Tilkynningaferill</t>
+          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni Upphefja Prófaðu Premium á 0 USD YouTube Kids Tilkynningaferill</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV Hype YouTube Premium YouTube Kids Segnalazioni</t>
+          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV Hype Prova Premium a 0 $ YouTube Kids Segnalazioni</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides Popularizēšana YouTube Premium YouTube Kids Ziņošanas vēsture</t>
+          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides Popularizēšana Izmēģiniet Premium par 0 USD YouTube Kids Ziņošanas vēsture</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV Pagyrimai YouTube Premium YouTube Kids Pranešimų istorija</t>
+          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV Pagyrimai Išbandykite „Premium“ už 0 USD YouTube Kids Pranešimų istorija</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé Hájpolás YouTube Premium YouTube Kids Bejelentési előzmények</t>
+          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé Hájpolás Díjmentes Premium YouTube Kids Bejelentési előzmények</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv Hype YouTube Premium YouTube Kids Rapportagegeschiedenis</t>
+          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv Hype Probeer Premium voor $ 0 YouTube Kids Rapportagegeschiedenis</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV Podbijanie YouTube Premium YouTube Kids Historia zgłoszeń</t>
+          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV Podbijanie Premium bez opłat YouTube Kids Historia zgłoszeń</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV Hype YouTube Premium YouTube Kids Histórico de denúncias</t>
+          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV Hype Experimente o Premium por 0 € YouTube Kids Histórico de denúncias</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV Hype YouTube Premium YouTube Kids Histórico de denúncias</t>
+          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV Hype Teste o Premium por US$ 0 YouTube Kids Histórico de denúncias</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni Popullarizo YouTube Premium YouTube Kids Historiku i raportimeve</t>
+          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni Popullarizo Provo Premium: 0 USD YouTube Kids Historiku i raportimeve</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV Izražanje navdušenja YouTube Premium YouTube Kids Zgodovina poročil</t>
+          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV Izražanje navdušenja Premium za 0 USD YouTube Kids Zgodovina poročil</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV Hypetys YouTube Premium YouTube Kids Ilmoitushistoria</t>
+          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV Hypetys Kokeile maksutta YouTube Kids Ilmoitushistoria</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv Hajp YouTube Premium YouTube Kids Rapporthistorik</t>
+          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv Hajp Få Premium för 0 USD YouTube Kids Rapporthistorik</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình Khuấy động YouTube Premium YouTube Kids Nhật ký báo cáo</t>
+          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình Khuấy động Thử Premium miễn phí YouTube Kids Nhật ký báo cáo</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV Hype YouTube Premium YouTube Kids İçerik bildirme geçmişi</t>
+          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV Hype Ücretsiz Premium YouTube Kids İçerik bildirme geçmişi</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы Галасаванне YouTube Premium YouTube Kids Гісторыя скаргаў</t>
+          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы Галасаванне Паспрабаваць Premium бясплатна YouTube Kids Гісторыя скаргаў</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания Хайп YouTube Premium YouTube Kids Подадени сигнали</t>
+          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания Хайп Premium за 0,00 EUR YouTube Kids Подадени сигнали</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы Хайп YouTube Premium YouTube Детям Жалобы</t>
+          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы Хайп Premium бесплатно YouTube Детям Жалобы</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали Голосування YouTube Premium YouTube Kids Історія скарг</t>
+          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали Голосування Premium безкоштовно YouTube Kids Історія скарг</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές Hype YouTube Premium YouTube Kids Ιστορικό αναφορών</t>
+          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές Hype Δοκιμαστε το Premium με 0 $ YouTube Kids Ιστορικό αναφορών</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ Հայփել YouTube Premium YouTube Kids Բողոքների պատմություն</t>
+          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ Հայփել Փորձեք Premium-ը անվճար YouTube Kids Բողոքների պատմություն</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה הייפ YouTube Premium YouTube Kids היסטוריית הדיווחים</t>
+          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה הייפ מינוי Premium ב-0$ YouTube Kids היסטוריית הדיווחים</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية التشجيع YouTube Premium YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
+          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية التشجيع Premium مجانًا YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون هیجان‌افزایی YouTube Premium YouTube Kids سابقه گزارش</t>
+          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون هیجان‌افزایی Premium با ۰ دلار YouTube Kids سابقه گزارش</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो हाइप YouTube Premium YouTube Kids शिकायतों का डेटा</t>
+          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो हाइप बिना किसी शुल्क के Premium आज़माएं YouTube Kids शिकायतों का डेटा</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি হাইপ YouTube Premium YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
+          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি হাইপ $০ দিয়ে Premium ব্যবহার করে দেখুন YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ ਹਾਈਪ ਕਰੋ YouTube Premium YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
+          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ ਹਾਈਪ ਕਰੋ $0 ਵਿੱਚ Premium ਅਜ਼ਮਾਓ YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી હાઇપ YouTube Premium YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
+          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી હાઇપ $0માં Premium અજમાવો YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் ஹைப் YouTube Premium YouTube Kids புகார் வரலாறு</t>
+          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் ஹைப் $0க்கு Premium பயன்படுத்திப் பார்க்கலாம் YouTube Kids புகார் வரலாறு</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ హైప్ YouTube Premium YouTube Kids రిపోర్టుల హిస్టరీ</t>
+          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ హైప్ $0కి Premium ట్రై చేయండి YouTube Kids రిపోర్టుల హిస్టరీ</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 粉丝热推 YouTube Premium YouTube Kids 举报记录</t>
+          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 粉丝热推 免费试用 Premium YouTube Kids 举报记录</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 粉絲熱推 YouTube Premium YouTube Kids 檢舉記錄</t>
+          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 粉絲熱推 免付費試用 Premium YouTube Kids 檢舉記錄</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 粉絲推介 YouTube Premium YouTube Kids 舉報記錄</t>
+          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 粉絲推介 免費試用 Premium YouTube Kids 舉報記錄</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 ハイプ YouTube Premium YouTube Kids 報告履歴</t>
+          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 ハイプ Premium を無料体験 YouTube Kids 報告履歴</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV 하이프 YouTube Premium YouTube Kids 신고 기록</t>
+          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV 하이프 Premium을 무료로 체험하세요 YouTube Kids 신고 기록</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding the updated data sheet , making changes to the gen util and tests class
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
@@ -8,9 +8,454 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="verifyingSideMenuLanguageAsInSe" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="147">
+  <si>
+    <t>slot</t>
+  </si>
+  <si>
+    <t>premium</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV {slot} {premium} YouTube Kids Aangeegeskiedenis</t>
+  </si>
+  <si>
+    <t>Regstreeks || Ophef || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Probeer Premium vir $0</t>
+  </si>
+  <si>
+    <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV {slot} {premium} YouTube Kids Xəbər tarixçəsi</t>
+  </si>
+  <si>
+    <t>Canlı || Hayp || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || 0$-a Premium sınayın</t>
+  </si>
+  <si>
+    <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV {slot} {premium} YouTube Kids Histori laporan</t>
+  </si>
+  <si>
+    <t>Live || Beri hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Coba Premium $0</t>
+  </si>
+  <si>
+    <t>Početna stranica Shorts Pretplate Vi Historija Muzika Filmovi i TV {slot} {premium} YouTube Kids Historija prijava</t>
+  </si>
+  <si>
+    <t>Uživo || Poticanje interesovanja || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Isprobajte Premium za 0 USD</t>
+  </si>
+  <si>
+    <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió {slot} {premium} YouTube Kids Historial d'informes</t>
+  </si>
+  <si>
+    <t>En directe || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Prova Premium per 0 €</t>
+  </si>
+  <si>
+    <t>Start Shorts Abonnementer Dig Historik Musik Film og tv {slot} {premium} YouTube Kids Rapporteringshistorik</t>
+  </si>
+  <si>
+    <t>Live || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium for 0 USD</t>
+  </si>
+  <si>
+    <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows {slot} {premium} YouTube Kids Meldeverlauf</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium kostenlos ausprobieren</t>
+  </si>
+  <si>
+    <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad {slot} {premium} YouTube Kids Teavituste ajalugu</t>
+  </si>
+  <si>
+    <t>Otse || Haipimine || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium 0 dollariga</t>
+  </si>
+  <si>
+    <t>Home Shorts Subscriptions You History Music Movies &amp; TV {slot} {premium} YouTube Kids Report history</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Try Premium for $0</t>
+  </si>
+  <si>
+    <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series {slot} {premium} YouTube Kids Historial de denuncias</t>
+  </si>
+  <si>
+    <t>En directo || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Probar Premium sin coste</t>
+  </si>
+  <si>
+    <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV {slot} {premium} YouTube Kids Historial de denuncias</t>
+  </si>
+  <si>
+    <t>En vivo || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium por USD 0</t>
+  </si>
+  <si>
+    <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak {slot} {premium} YouTube Kids Salaketa-historia</t>
+  </si>
+  <si>
+    <t>Zuzenean || Ikusmin-adierazpenak || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Probatu Premium 0 dolarrean</t>
+  </si>
+  <si>
+    <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV {slot} {premium} YouTube Kids Signalements</t>
+  </si>
+  <si>
+    <t>Direct || Boost || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Essayez Premium pour 0 $</t>
+  </si>
+  <si>
+    <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision {slot} {premium} YouTube Kids Historique des rapports</t>
+  </si>
+  <si>
+    <t>Jeux vidéo || Applaudissement || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Essayez Premium pour 0 USD</t>
+  </si>
+  <si>
+    <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija {slot} {premium} YouTube Kids Povijest prijava</t>
+  </si>
+  <si>
+    <t>Uživo || Razglašavanje || (none)</t>
+  </si>
+  <si>
+    <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni {slot} {premium} YouTube Kids Tilkynningaferill</t>
+  </si>
+  <si>
+    <t>Í beinni || Upphefja || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Prófaðu Premium á 0 USD</t>
+  </si>
+  <si>
+    <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV {slot} {premium} YouTube Kids Segnalazioni</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Prova Premium a 0 $</t>
+  </si>
+  <si>
+    <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides {slot} {premium} YouTube Kids Ziņošanas vēsture</t>
+  </si>
+  <si>
+    <t>Tiešraide || Popularizēšana || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Izmēģiniet Premium par 0 USD</t>
+  </si>
+  <si>
+    <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV {slot} {premium} YouTube Kids Pranešimų istorija</t>
+  </si>
+  <si>
+    <t>Tiesiogiai || Pagyrimai || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Išbandykite „Premium“ už 0 USD</t>
+  </si>
+  <si>
+    <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé {slot} {premium} YouTube Kids Bejelentési előzmények</t>
+  </si>
+  <si>
+    <t>Élő || Hájpolás || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Díjmentes Premium</t>
+  </si>
+  <si>
+    <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv {slot} {premium} YouTube Kids Rapportagegeschiedenis</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Probeer Premium voor $ 0</t>
+  </si>
+  <si>
+    <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV {slot} {premium} YouTube Kids Historia zgłoszeń</t>
+  </si>
+  <si>
+    <t>Na żywo || Podbijanie || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium bez opłat</t>
+  </si>
+  <si>
+    <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV {slot} {premium} YouTube Kids Histórico de denúncias</t>
+  </si>
+  <si>
+    <t>Em direto || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Experimente o Premium por 0 €</t>
+  </si>
+  <si>
+    <t>Início Shorts Inscrições Você Histórico Música Filmes e TV {slot} {premium} YouTube Kids Histórico de denúncias</t>
+  </si>
+  <si>
+    <t>Ao vivo || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Teste o Premium por US$ 0</t>
+  </si>
+  <si>
+    <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni {slot} {premium} YouTube Kids Historiku i raportimeve</t>
+  </si>
+  <si>
+    <t>Drejtpërdrejt || Popullarizo || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Provo Premium: 0 USD</t>
+  </si>
+  <si>
+    <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV {slot} {premium} YouTube Kids Zgodovina poročil</t>
+  </si>
+  <si>
+    <t>V živo || Izražanje navdušenja || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium za 0 USD</t>
+  </si>
+  <si>
+    <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV {slot} {premium} YouTube Kids Ilmoitushistoria</t>
+  </si>
+  <si>
+    <t>Livetapahtumat || Hypetys || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Kokeile maksutta</t>
+  </si>
+  <si>
+    <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv {slot} {premium} YouTube Kids Rapporthistorik</t>
+  </si>
+  <si>
+    <t>Live || Hajp || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Få Premium för 0 USD</t>
+  </si>
+  <si>
+    <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình {slot} {premium} YouTube Kids Nhật ký báo cáo</t>
+  </si>
+  <si>
+    <t>Trực tiếp || Khuấy động || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Thử Premium miễn phí</t>
+  </si>
+  <si>
+    <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV {slot} {premium} YouTube Kids Içerik bildirme geçmişi</t>
+  </si>
+  <si>
+    <t>Canlı || Hype || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Ücretsiz Premium</t>
+  </si>
+  <si>
+    <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы {slot} {premium} YouTube Kids Гісторыя скаргаў</t>
+  </si>
+  <si>
+    <t>У жывым эфіры || Галасаванне || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Паспрабаваць Premium бясплатна</t>
+  </si>
+  <si>
+    <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания {slot} {premium} YouTube Kids Подадени сигнали</t>
+  </si>
+  <si>
+    <t>На живо || Хайп || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium за 0,00 EUR</t>
+  </si>
+  <si>
+    <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы {slot} {premium} YouTube Детям Жалобы</t>
+  </si>
+  <si>
+    <t>Трансляции || Хайп || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium бесплатно</t>
+  </si>
+  <si>
+    <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали {slot} {premium} YouTube Kids Історія скарг</t>
+  </si>
+  <si>
+    <t>Прямі трансляції || Голосування || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium безкоштовно</t>
+  </si>
+  <si>
+    <t>Αρχικη Shorts Εγγραφες Εσεις Ιστορικο Μουσικη Ταινιες και τηλεοπτικες εκπομπες {slot} {premium} YouTube Kids Ιστορικο αναφορων</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Δοκιμαστε το Premium με 0 $</t>
+  </si>
+  <si>
+    <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ {slot} {premium} YouTube Kids Բողոքների պատմություն</t>
+  </si>
+  <si>
+    <t>Ուղիղ հեռարձակում || Հայփել || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Փորձեք Premium-ը անվճար</t>
+  </si>
+  <si>
+    <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה {slot} {premium} YouTube Kids היסטוריית הדיווחים</t>
+  </si>
+  <si>
+    <t>בשידור חי || הייפ || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || מינוי Premium ב-0$</t>
+  </si>
+  <si>
+    <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية {slot} {premium} YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
+  </si>
+  <si>
+    <t>بث مباشر || التشجيع || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium مجانًا</t>
+  </si>
+  <si>
+    <t>صفحه اصلی کوتهویدیوها اشتراکها شما سابقه موسیقی فیلم و تلویزیون {slot} {premium} YouTube Kids سابقه گزارش</t>
+  </si>
+  <si>
+    <t>زنده || هیجانافزایی || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium با ۰ دلار</t>
+  </si>
+  <si>
+    <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो {slot} {premium} YouTube Kids शिकायतों का डेटा</t>
+  </si>
+  <si>
+    <t>लाइव || हाइप || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || बिना किसी शुल्क के Premium आज़माएं</t>
+  </si>
+  <si>
+    <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি {slot} {premium} YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
+  </si>
+  <si>
+    <t>লাইভ || হাইপ || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || $০ দিয়ে Premium ব্যবহার করে দেখুন</t>
+  </si>
+  <si>
+    <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ {slot} {premium} YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
+  </si>
+  <si>
+    <t>ਲਾਈਵ || ਹਾਈਪ ਕਰੋ || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || $0 ਵਿੱਚ Premium ਅਜ਼ਮਾਓ</t>
+  </si>
+  <si>
+    <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી {slot} {premium} YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
+  </si>
+  <si>
+    <t>લાઇવ || હાઇપ || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || $0માં Premium અજમાવો</t>
+  </si>
+  <si>
+    <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் {slot} {premium} YouTube Kids புகார் வரலாறு</t>
+  </si>
+  <si>
+    <t>நேரலை || ஹைப் || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || $0க்கு Premium பயன்படுத்திப் பார்க்கலாம்</t>
+  </si>
+  <si>
+    <t>మొదటి ట్యాబ్ Shorts సబ్స్క్రిప్షన్లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ {slot} {premium} YouTube Kids రిపోర్టుల హిస్టరీ</t>
+  </si>
+  <si>
+    <t>లైవ్ || హైప్ || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || $0కి Premium ట్రై చేయండి</t>
+  </si>
+  <si>
+    <t>首页 Shorts 订阅 我 历史记录 音乐 影视 {slot} {premium} YouTube Kids 举报记录</t>
+  </si>
+  <si>
+    <t>直播 || 粉丝热推 || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || 免费试用 Premium</t>
+  </si>
+  <si>
+    <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 {slot} {premium} YouTube Kids 檢舉記錄</t>
+  </si>
+  <si>
+    <t>直播 || 粉絲熱推 || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || 免付費試用 Premium</t>
+  </si>
+  <si>
+    <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 {slot} {premium} YouTube Kids 舉報記錄</t>
+  </si>
+  <si>
+    <t>直播 || 粉絲推介 || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || 免費試用 Premium</t>
+  </si>
+  <si>
+    <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 {slot} {premium} YouTube Kids 報告履歴</t>
+  </si>
+  <si>
+    <t>ライブ || ハイプ || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium を無料体験</t>
+  </si>
+  <si>
+    <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV {slot} {premium} YouTube Kids 신고 기록</t>
+  </si>
+  <si>
+    <t>라이브 || 하이프 || (none)</t>
+  </si>
+  <si>
+    <t>YouTube Premium || Premium을 무료로 체험하세요</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -427,15 +872,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="36.33203125" customWidth="1" min="1" max="1"/>
-    <col width="104.5546875" customWidth="1" style="1" min="2" max="2"/>
+    <col min="1" max="1" customWidth="true" width="36.33203125"/>
+    <col min="2" max="2" customWidth="true" style="1" width="104.5546875"/>
+    <col min="3" max="3" width="40.0" customWidth="true"/>
+    <col min="4" max="4" width="40.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>Applied Language</t>
         </is>
@@ -445,641 +892,859 @@
           <t>Expected Data</t>
         </is>
       </c>
+      <c r="C1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" ht="28.8" customHeight="1">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>Afrikaans</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV Ophef Probeer Premium vir $0 YouTube Kids Aangeegeskiedenis</t>
-        </is>
+      <c r="B2" t="s" s="1">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s" s="1">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>5</v>
       </c>
     </row>
     <row r="3" ht="28.8" customHeight="1">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr" s="0">
         <is>
           <t>Azərbaycan</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Ev Shorts Abunəliklər Siz Tarixçə Musiqi Film və TV Hayp 0$-a Premium sınayın YouTube Kids Xəbər tarixçəsi</t>
-        </is>
+      <c r="B3" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s" s="1">
+        <v>8</v>
       </c>
     </row>
     <row r="4" ht="28.8" customHeight="1">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="inlineStr" s="0">
         <is>
           <t>Bahasa Indonesia</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Beranda Shorts Subscription Anda Histori Musik Film &amp; TV Beri hype Coba Premium $0 YouTube Kids Histori laporan</t>
-        </is>
+      <c r="B4" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s" s="1">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s" s="1">
+        <v>11</v>
       </c>
     </row>
     <row r="5" ht="28.8" customHeight="1">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="inlineStr" s="0">
         <is>
           <t>Bosanski</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Početna stranica Shorts Pretplate Vi Hi‪storija Muzika Filmovi i TV Poticanje interesovanja Isprobajte Premium za 0 USD YouTube Kids Historija prijava</t>
-        </is>
+      <c r="B5" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="6" ht="28.8" customHeight="1">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="inlineStr" s="0">
         <is>
           <t>Català</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Inici Shorts Subscripcions Tu Historial Música Pel·lícules i televisió Hype Prova Premium per 0 € YouTube Kids Historial d'informes</t>
-        </is>
+      <c r="B6" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s" s="1">
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="28.8" customHeight="1">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="inlineStr" s="0">
         <is>
           <t>Dansk</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Start Shorts Abonnementer Dig Historik Musik Film og tv Hype Premium for 0 USD YouTube Kids Rapporteringshistorik</t>
-        </is>
+      <c r="B7" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s" s="1">
+        <v>20</v>
       </c>
     </row>
     <row r="8" ht="28.8" customHeight="1">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="inlineStr" s="0">
         <is>
           <t>Deutsch</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Startseite Shorts Abos Mein YouTube Verlauf Musik Filme &amp; Shows Hype Premium kostenlos ausprobieren YouTube Kids Meldeverlauf</t>
-        </is>
+      <c r="B8" t="s" s="1">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s" s="1">
+        <v>22</v>
       </c>
     </row>
     <row r="9" ht="28.8" customHeight="1">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr" s="0">
         <is>
           <t>Eesti</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Avaleht Shorts Tellimused Teie Ajalugu Muusika Filmid ja telesarjad Haipimine Premium 0 dollariga YouTube Kids Teavituste ajalugu</t>
-        </is>
+      <c r="B9" t="s" s="1">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s" s="1">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s" s="1">
+        <v>25</v>
       </c>
     </row>
     <row r="10" ht="28.8" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr" s="0">
         <is>
           <t>English (India)</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype Try Premium for $0 YouTube Kids Report history</t>
-        </is>
+      <c r="B10" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s" s="1">
+        <v>27</v>
       </c>
     </row>
     <row r="11" ht="28.8" customHeight="1">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="inlineStr" s="0">
         <is>
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype Try Premium for $0 YouTube Kids Report history</t>
-        </is>
+      <c r="B11" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D11" t="s" s="1">
+        <v>27</v>
       </c>
     </row>
     <row r="12" ht="28.8" customHeight="1">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="inlineStr" s="0">
         <is>
           <t>English (US)</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Home Shorts Subscriptions You History Music Movies &amp; TV Hype Try Premium for $0 YouTube Kids Report history</t>
-        </is>
+      <c r="B12" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s" s="1">
+        <v>27</v>
       </c>
     </row>
     <row r="13" ht="28.8" customHeight="1">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="inlineStr" s="0">
         <is>
           <t>Español (España)</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>Inicio Shorts Suscripciones Tú Historial Música Películas y series Hype Probar Premium sin coste YouTube Kids Historial de denuncias</t>
-        </is>
+      <c r="B13" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s" s="1">
+        <v>30</v>
       </c>
     </row>
     <row r="14" ht="28.8" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="inlineStr" s="0">
         <is>
           <t>Español (Latinoamérica)</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype Premium por USD 0 YouTube Kids Historial de denuncias</t>
-        </is>
+      <c r="B14" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s" s="1">
+        <v>33</v>
       </c>
     </row>
     <row r="15" ht="28.8" customHeight="1">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="inlineStr" s="0">
         <is>
           <t>Español (US)</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Principal Shorts Suscripciones Tú Historial Música Películas y TV Hype Premium por USD 0 YouTube Kids Historial de denuncias</t>
-        </is>
+      <c r="B15" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="D15" t="s" s="1">
+        <v>33</v>
       </c>
     </row>
     <row r="16" ht="28.8" customHeight="1">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="inlineStr" s="0">
         <is>
           <t>Euskara</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>Orri nagusia Shorts Harpidetzak Zu Historia Musika Filmak eta saioak Ikusmin-adierazpenak Probatu Premium 0 dolarrean YouTube Kids Salaketa-historia</t>
-        </is>
+      <c r="B16" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="D16" t="s" s="1">
+        <v>36</v>
       </c>
     </row>
     <row r="17" ht="28.8" customHeight="1">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="inlineStr" s="0">
         <is>
           <t>Français</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et séries TV Boost Essayez Premium pour 0 $ YouTube Kids Signalements</t>
-        </is>
+      <c r="B17" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="C17" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s" s="1">
+        <v>39</v>
       </c>
     </row>
     <row r="18" ht="28.8" customHeight="1">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="inlineStr" s="0">
         <is>
           <t>Français (Canada)</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>Accueil Shorts Abonnements Vous Historique Musique Films et émissions de télévision Applaudissement Essayez Premium pour 0 USD YouTube Kids Historique des rapports</t>
-        </is>
+      <c r="B18" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s" s="1">
+        <v>41</v>
+      </c>
+      <c r="D18" t="s" s="1">
+        <v>42</v>
       </c>
     </row>
     <row r="19" ht="28.8" customHeight="1">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="inlineStr" s="0">
         <is>
           <t>Hrvatski</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Početna Shorts Pretplate Moje Povijest Glazba Filmovi i televizija Razglašavanje Isprobajte Premium za 0 USD YouTube Kids Povijest prijava</t>
-        </is>
+      <c r="B19" t="s" s="1">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s" s="1">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="20" ht="28.8" customHeight="1">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="inlineStr" s="0">
         <is>
           <t>Íslenska</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Heim Shorts Áskriftir Þú Ferill Tónlist Kvikmyndir og sjónvarpsefni Upphefja Prófaðu Premium á 0 USD YouTube Kids Tilkynningaferill</t>
-        </is>
+      <c r="B20" t="s" s="1">
+        <v>45</v>
+      </c>
+      <c r="C20" t="s" s="1">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s" s="1">
+        <v>47</v>
       </c>
     </row>
     <row r="21" ht="28.8" customHeight="1">
-      <c r="A21" t="inlineStr">
+      <c r="A21" t="inlineStr" s="0">
         <is>
           <t>Italiano</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Home Shorts Iscrizioni Tu Cronologia Musica Film e TV Hype Prova Premium a 0 $ YouTube Kids Segnalazioni</t>
-        </is>
+      <c r="B21" t="s" s="1">
+        <v>48</v>
+      </c>
+      <c r="C21" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D21" t="s" s="1">
+        <v>49</v>
       </c>
     </row>
     <row r="22" ht="28.8" customHeight="1">
-      <c r="A22" t="inlineStr">
+      <c r="A22" t="inlineStr" s="0">
         <is>
           <t>Latviešu valoda</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Sākums Shorts Abonementi Jūs Vēsture Mūzika Filmas un TV pārraides Popularizēšana Izmēģiniet Premium par 0 USD YouTube Kids Ziņošanas vēsture</t>
-        </is>
+      <c r="B22" t="s" s="1">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s" s="1">
+        <v>51</v>
+      </c>
+      <c r="D22" t="s" s="1">
+        <v>52</v>
       </c>
     </row>
     <row r="23" ht="28.8" customHeight="1">
-      <c r="A23" t="inlineStr">
+      <c r="A23" t="inlineStr" s="0">
         <is>
           <t>Lietuvių</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>Pagrindinis Shorts Prenumeratos Jūs Istorija Muzika Filmai ir TV Pagyrimai Išbandykite „Premium“ už 0 USD YouTube Kids Pranešimų istorija</t>
-        </is>
+      <c r="B23" t="s" s="1">
+        <v>53</v>
+      </c>
+      <c r="C23" t="s" s="1">
+        <v>54</v>
+      </c>
+      <c r="D23" t="s" s="1">
+        <v>55</v>
       </c>
     </row>
     <row r="24" ht="28.8" customHeight="1">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="inlineStr" s="0">
         <is>
           <t>Magyar</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>Kezdőlap Shorts Feliratkozások Te Előzmények Zene Film és tévé Hájpolás Díjmentes Premium YouTube Kids Bejelentési előzmények</t>
-        </is>
+      <c r="B24" t="s" s="1">
+        <v>56</v>
+      </c>
+      <c r="C24" t="s" s="1">
+        <v>57</v>
+      </c>
+      <c r="D24" t="s" s="1">
+        <v>58</v>
       </c>
     </row>
     <row r="25" ht="28.8" customHeight="1">
-      <c r="A25" t="inlineStr">
+      <c r="A25" t="inlineStr" s="0">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>Home Shorts Abonnementen Jij Geschiedenis Muziek Films en tv Hype Probeer Premium voor $ 0 YouTube Kids Rapportagegeschiedenis</t>
-        </is>
+      <c r="B25" t="s" s="1">
+        <v>59</v>
+      </c>
+      <c r="C25" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D25" t="s" s="1">
+        <v>60</v>
       </c>
     </row>
     <row r="26" ht="28.8" customHeight="1">
-      <c r="A26" t="inlineStr">
+      <c r="A26" t="inlineStr" s="0">
         <is>
           <t>Polski</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>Główna Shorts Subskrypcje Ty Historia Muzyka Filmy i TV Podbijanie Premium bez opłat YouTube Kids Historia zgłoszeń</t>
-        </is>
+      <c r="B26" t="s" s="1">
+        <v>61</v>
+      </c>
+      <c r="C26" t="s" s="1">
+        <v>62</v>
+      </c>
+      <c r="D26" t="s" s="1">
+        <v>63</v>
       </c>
     </row>
     <row r="27" ht="28.8" customHeight="1">
-      <c r="A27" t="inlineStr">
+      <c r="A27" t="inlineStr" s="0">
         <is>
           <t>Português</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>Início Shorts Subscrições Eu Histórico Música Filmes e TV Hype Experimente o Premium por 0 € YouTube Kids Histórico de denúncias</t>
-        </is>
+      <c r="B27" t="s" s="1">
+        <v>64</v>
+      </c>
+      <c r="C27" t="s" s="1">
+        <v>65</v>
+      </c>
+      <c r="D27" t="s" s="1">
+        <v>66</v>
       </c>
     </row>
     <row r="28" ht="28.8" customHeight="1">
-      <c r="A28" t="inlineStr">
+      <c r="A28" t="inlineStr" s="0">
         <is>
           <t>Português (Brasil)</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Início Shorts Inscrições Você Histórico Música Filmes e TV Hype Teste o Premium por US$ 0 YouTube Kids Histórico de denúncias</t>
-        </is>
+      <c r="B28" t="s" s="1">
+        <v>67</v>
+      </c>
+      <c r="C28" t="s" s="1">
+        <v>68</v>
+      </c>
+      <c r="D28" t="s" s="1">
+        <v>69</v>
       </c>
     </row>
     <row r="29" ht="28.8" customHeight="1">
-      <c r="A29" t="inlineStr">
+      <c r="A29" t="inlineStr" s="0">
         <is>
           <t>Shqip</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>Faqja e parë Shorts Abonimet Ti Historiku Muzikë Filmat dhe televizioni Popullarizo Provo Premium: 0 USD YouTube Kids Historiku i raportimeve</t>
-        </is>
+      <c r="B29" t="s" s="1">
+        <v>70</v>
+      </c>
+      <c r="C29" t="s" s="1">
+        <v>71</v>
+      </c>
+      <c r="D29" t="s" s="1">
+        <v>72</v>
       </c>
     </row>
     <row r="30" ht="28.8" customHeight="1">
-      <c r="A30" t="inlineStr">
+      <c r="A30" t="inlineStr" s="0">
         <is>
           <t>Slovenščina</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
-        <is>
-          <t>Domača stran Kratki videoposnetki Naročnine Vi Zgodovina Glasba Filmi in TV Izražanje navdušenja Premium za 0 USD YouTube Kids Zgodovina poročil</t>
-        </is>
+      <c r="B30" t="s" s="1">
+        <v>73</v>
+      </c>
+      <c r="C30" t="s" s="1">
+        <v>74</v>
+      </c>
+      <c r="D30" t="s" s="1">
+        <v>75</v>
       </c>
     </row>
     <row r="31" ht="28.8" customHeight="1">
-      <c r="A31" t="inlineStr">
+      <c r="A31" t="inlineStr" s="0">
         <is>
           <t>Suomi</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
-        <is>
-          <t>Koti Shorts Tilaukset Sinä Historia Musiikki Elokuvat ja TV Hypetys Kokeile maksutta YouTube Kids Ilmoitushistoria</t>
-        </is>
+      <c r="B31" t="s" s="1">
+        <v>76</v>
+      </c>
+      <c r="C31" t="s" s="1">
+        <v>77</v>
+      </c>
+      <c r="D31" t="s" s="1">
+        <v>78</v>
       </c>
     </row>
     <row r="32" ht="28.8" customHeight="1">
-      <c r="A32" t="inlineStr">
+      <c r="A32" t="inlineStr" s="0">
         <is>
           <t>Svenska</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t>Hem Shorts Prenumerationer Ditt YouTube Historik Musik Filmer och tv Hajp Få Premium för 0 USD YouTube Kids Rapporthistorik</t>
-        </is>
+      <c r="B32" t="s" s="1">
+        <v>79</v>
+      </c>
+      <c r="C32" t="s" s="1">
+        <v>80</v>
+      </c>
+      <c r="D32" t="s" s="1">
+        <v>81</v>
       </c>
     </row>
     <row r="33" ht="28.8" customHeight="1">
-      <c r="A33" t="inlineStr">
+      <c r="A33" t="inlineStr" s="0">
         <is>
           <t>Tiếng Việt</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
-        <is>
-          <t>Trang chủ Shorts Kênh đăng ký Bạn Video đã xem Âm nhạc Phim và truyền hình Khuấy động Thử Premium miễn phí YouTube Kids Nhật ký báo cáo</t>
-        </is>
+      <c r="B33" t="s" s="1">
+        <v>82</v>
+      </c>
+      <c r="C33" t="s" s="1">
+        <v>83</v>
+      </c>
+      <c r="D33" t="s" s="1">
+        <v>84</v>
       </c>
     </row>
     <row r="34" ht="28.8" customHeight="1">
-      <c r="A34" t="inlineStr">
+      <c r="A34" t="inlineStr" s="0">
         <is>
           <t>Türkçe</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
-        <is>
-          <t>Ana Sayfa Shorts Abonelikler Siz Geçmiş Müzik Filmler ve TV Hype Ücretsiz Premium YouTube Kids İçerik bildirme geçmişi</t>
-        </is>
+      <c r="B34" t="s" s="1">
+        <v>85</v>
+      </c>
+      <c r="C34" t="s" s="1">
+        <v>86</v>
+      </c>
+      <c r="D34" t="s" s="1">
+        <v>87</v>
       </c>
     </row>
     <row r="35" ht="28.8" customHeight="1">
-      <c r="A35" t="inlineStr">
+      <c r="A35" t="inlineStr" s="0">
         <is>
           <t>Беларуская</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
-        <is>
-          <t>Галоўная старонка Shorts Падпіскі Вы Гісторыя Музыка Фільмы і тэлеперадачы Галасаванне Паспрабаваць Premium бясплатна YouTube Kids Гісторыя скаргаў</t>
-        </is>
+      <c r="B35" t="s" s="1">
+        <v>88</v>
+      </c>
+      <c r="C35" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="D35" t="s" s="1">
+        <v>90</v>
       </c>
     </row>
     <row r="36" ht="28.8" customHeight="1">
-      <c r="A36" t="inlineStr">
+      <c r="A36" t="inlineStr" s="0">
         <is>
           <t>Български</t>
         </is>
       </c>
-      <c r="B36" s="1" t="inlineStr">
-        <is>
-          <t>Начало Shorts Абонаменти Вие История Музика Филми и телевизионни предавания Хайп Premium за 0,00 EUR YouTube Kids Подадени сигнали</t>
-        </is>
+      <c r="B36" t="s" s="1">
+        <v>91</v>
+      </c>
+      <c r="C36" t="s" s="1">
+        <v>92</v>
+      </c>
+      <c r="D36" t="s" s="1">
+        <v>93</v>
       </c>
     </row>
     <row r="37" ht="28.8" customHeight="1">
-      <c r="A37" t="inlineStr">
+      <c r="A37" t="inlineStr" s="0">
         <is>
           <t>Русский</t>
         </is>
       </c>
-      <c r="B37" s="1" t="inlineStr">
-        <is>
-          <t>Главная Shorts Подписки Вы История Музыка Фильмы и сериалы Хайп Premium бесплатно YouTube Детям Жалобы</t>
-        </is>
+      <c r="B37" t="s" s="1">
+        <v>94</v>
+      </c>
+      <c r="C37" t="s" s="1">
+        <v>95</v>
+      </c>
+      <c r="D37" t="s" s="1">
+        <v>96</v>
       </c>
     </row>
     <row r="38" ht="28.8" customHeight="1">
-      <c r="A38" t="inlineStr">
+      <c r="A38" t="inlineStr" s="0">
         <is>
           <t>Українська</t>
         </is>
       </c>
-      <c r="B38" s="1" t="inlineStr">
-        <is>
-          <t>Головна YouTube Shorts Підписки Ви Історія Музика Фільми й серіали Голосування Premium безкоштовно YouTube Kids Історія скарг</t>
-        </is>
+      <c r="B38" t="s" s="1">
+        <v>97</v>
+      </c>
+      <c r="C38" t="s" s="1">
+        <v>98</v>
+      </c>
+      <c r="D38" t="s" s="1">
+        <v>99</v>
       </c>
     </row>
     <row r="39" ht="28.8" customHeight="1">
-      <c r="A39" t="inlineStr">
+      <c r="A39" t="inlineStr" s="0">
         <is>
           <t>Ελληνικά</t>
         </is>
       </c>
-      <c r="B39" s="1" t="inlineStr">
-        <is>
-          <t>Αρχική Shorts Εγγραφές Εσείς Ιστορικό Μουσική Ταινίες και τηλεοπτικές εκπομπές Hype Δοκιμαστε το Premium με 0 $ YouTube Kids Ιστορικό αναφορών</t>
-        </is>
+      <c r="B39" t="s" s="1">
+        <v>100</v>
+      </c>
+      <c r="C39" t="s" s="1">
+        <v>19</v>
+      </c>
+      <c r="D39" t="s" s="1">
+        <v>101</v>
       </c>
     </row>
     <row r="40" ht="28.8" customHeight="1">
-      <c r="A40" t="inlineStr">
+      <c r="A40" t="inlineStr" s="0">
         <is>
           <t>Հայերեն</t>
         </is>
       </c>
-      <c r="B40" s="1" t="inlineStr">
-        <is>
-          <t>Սկիզբ Shorts Հետևում եմ Դուք Պատմություն Երաժշտություն Ֆիլմեր և սերիալներ Հայփել Փորձեք Premium-ը անվճար YouTube Kids Բողոքների պատմություն</t>
-        </is>
+      <c r="B40" t="s" s="1">
+        <v>102</v>
+      </c>
+      <c r="C40" t="s" s="1">
+        <v>103</v>
+      </c>
+      <c r="D40" t="s" s="1">
+        <v>104</v>
       </c>
     </row>
     <row r="41" ht="28.8" customHeight="1">
-      <c r="A41" t="inlineStr">
+      <c r="A41" t="inlineStr" s="0">
         <is>
           <t>עברית</t>
         </is>
       </c>
-      <c r="B41" s="1" t="inlineStr">
-        <is>
-          <t>דף הבית Shorts מינויים הדף שלי היסטוריה מוזיקה סרטים ותוכניות טלוויזיה הייפ מינוי Premium ב-0$ YouTube Kids היסטוריית הדיווחים</t>
-        </is>
+      <c r="B41" t="s" s="1">
+        <v>105</v>
+      </c>
+      <c r="C41" t="s" s="1">
+        <v>106</v>
+      </c>
+      <c r="D41" t="s" s="1">
+        <v>107</v>
       </c>
     </row>
     <row r="42" ht="28.8" customHeight="1">
-      <c r="A42" t="inlineStr">
+      <c r="A42" t="inlineStr" s="0">
         <is>
           <t>العربية</t>
         </is>
       </c>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>الصفحة الرئيسية Shorts الاشتراكات أنت السجلّ موسيقى أفلام وبرامج تلفزيونية التشجيع Premium مجانًا YouTube Kids سجلّ الإبلاغ عن المحتوى</t>
-        </is>
+      <c r="B42" t="s" s="1">
+        <v>108</v>
+      </c>
+      <c r="C42" t="s" s="1">
+        <v>109</v>
+      </c>
+      <c r="D42" t="s" s="1">
+        <v>110</v>
       </c>
     </row>
     <row r="43" ht="28.8" customHeight="1">
-      <c r="A43" t="inlineStr">
+      <c r="A43" t="inlineStr" s="0">
         <is>
           <t>فارسی</t>
         </is>
       </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>صفحه اصلی کوته‌ویدیوها اشتراک‌ها شما سابقه موسیقی فیلم و تلویزیون هیجان‌افزایی Premium با ۰ دلار YouTube Kids سابقه گزارش</t>
-        </is>
+      <c r="B43" t="s" s="1">
+        <v>111</v>
+      </c>
+      <c r="C43" t="s" s="1">
+        <v>112</v>
+      </c>
+      <c r="D43" t="s" s="1">
+        <v>113</v>
       </c>
     </row>
     <row r="44" ht="28.8" customHeight="1">
-      <c r="A44" t="inlineStr">
+      <c r="A44" t="inlineStr" s="0">
         <is>
           <t>हिन्दी</t>
         </is>
       </c>
-      <c r="B44" s="1" t="inlineStr">
-        <is>
-          <t>होम पेज Shorts सदस्यता आप देखे गए वीडियो संगीत फ़िल्में और टीवी शो हाइप बिना किसी शुल्क के Premium आज़माएं YouTube Kids शिकायतों का डेटा</t>
-        </is>
+      <c r="B44" t="s" s="1">
+        <v>114</v>
+      </c>
+      <c r="C44" t="s" s="1">
+        <v>115</v>
+      </c>
+      <c r="D44" t="s" s="1">
+        <v>116</v>
       </c>
     </row>
     <row r="45" ht="28.8" customHeight="1">
-      <c r="A45" t="inlineStr">
+      <c r="A45" t="inlineStr" s="0">
         <is>
           <t>বাংলা</t>
         </is>
       </c>
-      <c r="B45" s="1" t="inlineStr">
-        <is>
-          <t>হোম Shorts সাবস্ক্রিপশন আপনি ইতিহাস মিউজিক সিনেমা ও টিভি হাইপ $০ দিয়ে Premium ব্যবহার করে দেখুন YouTube Kids অভিযোগ জানানোর ইতিহাস</t>
-        </is>
+      <c r="B45" t="s" s="1">
+        <v>117</v>
+      </c>
+      <c r="C45" t="s" s="1">
+        <v>118</v>
+      </c>
+      <c r="D45" t="s" s="1">
+        <v>119</v>
       </c>
     </row>
     <row r="46" ht="28.8" customHeight="1">
-      <c r="A46" t="inlineStr">
+      <c r="A46" t="inlineStr" s="0">
         <is>
           <t>ਪੰਜਾਬੀ</t>
         </is>
       </c>
-      <c r="B46" s="1" t="inlineStr">
-        <is>
-          <t>ਹੋਮ Shorts ਸਬਸਕ੍ਰਿਪਸ਼ਨਾਂ ਤੁਸੀਂ ਇਤਿਹਾਸ ਸੰਗੀਤ ਫ਼ਿਲਮਾਂ ਅਤੇ ਟੀਵੀ ਹਾਈਪ ਕਰੋ $0 ਵਿੱਚ Premium ਅਜ਼ਮਾਓ YouTube Kids ਰਿਪੋਰਟ ਸੰਬੰਧੀ ਇਤਿਹਾਸ</t>
-        </is>
+      <c r="B46" t="s" s="1">
+        <v>120</v>
+      </c>
+      <c r="C46" t="s" s="1">
+        <v>121</v>
+      </c>
+      <c r="D46" t="s" s="1">
+        <v>122</v>
       </c>
     </row>
     <row r="47" ht="28.8" customHeight="1">
-      <c r="A47" t="inlineStr">
+      <c r="A47" t="inlineStr" s="0">
         <is>
           <t>ગુજરાતી</t>
         </is>
       </c>
-      <c r="B47" s="1" t="inlineStr">
-        <is>
-          <t>હોમ Shorts સબ્સ્ક્રિપ્શન તમે ઇતિહાસ સંગીત મૂવી અને ટીવી હાઇપ $0માં Premium અજમાવો YouTube Kids રિપોર્ટનો ઇતિહાસ</t>
-        </is>
+      <c r="B47" t="s" s="1">
+        <v>123</v>
+      </c>
+      <c r="C47" t="s" s="1">
+        <v>124</v>
+      </c>
+      <c r="D47" t="s" s="1">
+        <v>125</v>
       </c>
     </row>
     <row r="48" ht="28.8" customHeight="1">
-      <c r="A48" t="inlineStr">
+      <c r="A48" t="inlineStr" s="0">
         <is>
           <t>தமிழ்</t>
         </is>
       </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>முகப்பு Shorts சந்தாக்கள் நீங்கள் இதுவரை பார்த்தவை இசை திரைப்படங்கள் &amp; டிவி நிகழ்ச்சிகள் ஹைப் $0க்கு Premium பயன்படுத்திப் பார்க்கலாம் YouTube Kids புகார் வரலாறு</t>
-        </is>
+      <c r="B48" t="s" s="1">
+        <v>126</v>
+      </c>
+      <c r="C48" t="s" s="1">
+        <v>127</v>
+      </c>
+      <c r="D48" t="s" s="1">
+        <v>128</v>
       </c>
     </row>
     <row r="49" ht="28.8" customHeight="1">
-      <c r="A49" t="inlineStr">
+      <c r="A49" t="inlineStr" s="0">
         <is>
           <t>తెలుగు</t>
         </is>
       </c>
-      <c r="B49" s="1" t="inlineStr">
-        <is>
-          <t>మొదటి ట్యాబ్ Shorts సబ్‌స్క్రిప్షన్‌లు ఖాతా హిస్టరీ మ్యూజిక్ సినిమాలు &amp; టీవీ హైప్ $0కి Premium ట్రై చేయండి YouTube Kids రిపోర్టుల హిస్టరీ</t>
-        </is>
+      <c r="B49" t="s" s="1">
+        <v>129</v>
+      </c>
+      <c r="C49" t="s" s="1">
+        <v>130</v>
+      </c>
+      <c r="D49" t="s" s="1">
+        <v>131</v>
       </c>
     </row>
     <row r="50" ht="28.8" customHeight="1">
-      <c r="A50" t="inlineStr">
+      <c r="A50" t="inlineStr" s="0">
         <is>
           <t>中文 (简体)</t>
         </is>
       </c>
-      <c r="B50" s="1" t="inlineStr">
-        <is>
-          <t>首页 Shorts 订阅 我 历史记录 音乐 影视 粉丝热推 免费试用 Premium YouTube Kids 举报记录</t>
-        </is>
+      <c r="B50" t="s" s="1">
+        <v>132</v>
+      </c>
+      <c r="C50" t="s" s="1">
+        <v>133</v>
+      </c>
+      <c r="D50" t="s" s="1">
+        <v>134</v>
       </c>
     </row>
     <row r="51" ht="28.8" customHeight="1">
-      <c r="A51" t="inlineStr">
+      <c r="A51" t="inlineStr" s="0">
         <is>
           <t>中文 (繁體)</t>
         </is>
       </c>
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t>首頁 Shorts 訂閱內容 個人中心 觀看記錄 音樂 電影與電視節目 粉絲熱推 免付費試用 Premium YouTube Kids 檢舉記錄</t>
-        </is>
+      <c r="B51" t="s" s="1">
+        <v>135</v>
+      </c>
+      <c r="C51" t="s" s="1">
+        <v>136</v>
+      </c>
+      <c r="D51" t="s" s="1">
+        <v>137</v>
       </c>
     </row>
     <row r="52" ht="28.8" customHeight="1">
-      <c r="A52" t="inlineStr">
+      <c r="A52" t="inlineStr" s="0">
         <is>
           <t>中文 (香港)</t>
         </is>
       </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>主頁 Shorts 訂閱項目 個人中心 記錄 音樂 電影和電視節目 粉絲推介 免費試用 Premium YouTube Kids 舉報記錄</t>
-        </is>
+      <c r="B52" t="s" s="1">
+        <v>138</v>
+      </c>
+      <c r="C52" t="s" s="1">
+        <v>139</v>
+      </c>
+      <c r="D52" t="s" s="1">
+        <v>140</v>
       </c>
     </row>
     <row r="53" ht="28.8" customHeight="1">
-      <c r="A53" t="inlineStr">
+      <c r="A53" t="inlineStr" s="0">
         <is>
           <t>日本語</t>
         </is>
       </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>ホーム ショート 登録チャンネル マイページ 履歴 音楽 映画とテレビ番組 ハイプ Premium を無料体験 YouTube Kids 報告履歴</t>
-        </is>
+      <c r="B53" t="s" s="1">
+        <v>141</v>
+      </c>
+      <c r="C53" t="s" s="1">
+        <v>142</v>
+      </c>
+      <c r="D53" t="s" s="1">
+        <v>143</v>
       </c>
     </row>
     <row r="54" ht="28.8" customHeight="1">
-      <c r="A54" t="inlineStr">
+      <c r="A54" t="inlineStr" s="0">
         <is>
           <t>한국어</t>
         </is>
       </c>
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t>홈 Shorts 구독 내 페이지 기록 음악 영화 및 TV 하이프 Premium을 무료로 체험하세요 YouTube Kids 신고 기록</t>
-        </is>
+      <c r="B54" t="s" s="1">
+        <v>144</v>
+      </c>
+      <c r="C54" t="s" s="1">
+        <v>145</v>
+      </c>
+      <c r="D54" t="s" s="1">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
trying the ci gate check
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
@@ -1,28 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sagar\youtube-multi-language-ui-validator-automation\yt_multi_language_ui_validator\src\main\resources\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E0BBB2A-932D-4207-870B-5BB5B9B5736E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="verifyingSideMenuLanguageAsInSe" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="verifyingSideMenuLanguageAsInSe" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="147">
-  <si>
-    <t>slot</t>
-  </si>
-  <si>
-    <t>premium</t>
-  </si>
-  <si>
-    <t/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="199">
   <si>
     <t>Tuis Kortvideo's Intekeninge Myne Geskiedenis Musiek Flieks en TV {slot} {premium} YouTube Kids Aangeegeskiedenis</t>
   </si>
@@ -454,25 +452,189 @@
   </si>
   <si>
     <t>YouTube Premium || Premium을 무료로 체험하세요</t>
+  </si>
+  <si>
+    <t>Applied Language</t>
+  </si>
+  <si>
+    <t>Expected Data</t>
+  </si>
+  <si>
+    <t>Afrikaans</t>
+  </si>
+  <si>
+    <t>Azərbaycan</t>
+  </si>
+  <si>
+    <t>Bahasa Indonesia</t>
+  </si>
+  <si>
+    <t>Bosanski</t>
+  </si>
+  <si>
+    <t>Català</t>
+  </si>
+  <si>
+    <t>Dansk</t>
+  </si>
+  <si>
+    <t>Deutsch</t>
+  </si>
+  <si>
+    <t>Eesti</t>
+  </si>
+  <si>
+    <t>English (India)</t>
+  </si>
+  <si>
+    <t>English (UK)</t>
+  </si>
+  <si>
+    <t>English (US)</t>
+  </si>
+  <si>
+    <t>Español (España)</t>
+  </si>
+  <si>
+    <t>Español (Latinoamérica)</t>
+  </si>
+  <si>
+    <t>Español (US)</t>
+  </si>
+  <si>
+    <t>Euskara</t>
+  </si>
+  <si>
+    <t>Français</t>
+  </si>
+  <si>
+    <t>Français (Canada)</t>
+  </si>
+  <si>
+    <t>Hrvatski</t>
+  </si>
+  <si>
+    <t>Íslenska</t>
+  </si>
+  <si>
+    <t>Italiano</t>
+  </si>
+  <si>
+    <t>Latviešu valoda</t>
+  </si>
+  <si>
+    <t>Lietuvių</t>
+  </si>
+  <si>
+    <t>Magyar</t>
+  </si>
+  <si>
+    <t>Nederlands</t>
+  </si>
+  <si>
+    <t>Polski</t>
+  </si>
+  <si>
+    <t>Português</t>
+  </si>
+  <si>
+    <t>Português (Brasil)</t>
+  </si>
+  <si>
+    <t>Shqip</t>
+  </si>
+  <si>
+    <t>Slovenščina</t>
+  </si>
+  <si>
+    <t>Suomi</t>
+  </si>
+  <si>
+    <t>Svenska</t>
+  </si>
+  <si>
+    <t>Tiếng Việt</t>
+  </si>
+  <si>
+    <t>Türkçe</t>
+  </si>
+  <si>
+    <t>Беларуская</t>
+  </si>
+  <si>
+    <t>Български</t>
+  </si>
+  <si>
+    <t>Русский</t>
+  </si>
+  <si>
+    <t>Українська</t>
+  </si>
+  <si>
+    <t>Ελληνικά</t>
+  </si>
+  <si>
+    <t>Հայերեն</t>
+  </si>
+  <si>
+    <t>עברית</t>
+  </si>
+  <si>
+    <t>العربية</t>
+  </si>
+  <si>
+    <t>فارسی</t>
+  </si>
+  <si>
+    <t>हिन्दी</t>
+  </si>
+  <si>
+    <t>বাংলা</t>
+  </si>
+  <si>
+    <t>ਪੰਜਾਬੀ</t>
+  </si>
+  <si>
+    <t>ગુજરાતી</t>
+  </si>
+  <si>
+    <t>தமிழ்</t>
+  </si>
+  <si>
+    <t>తెలుగు</t>
+  </si>
+  <si>
+    <t>中文 (简体)</t>
+  </si>
+  <si>
+    <t>中文 (繁體)</t>
+  </si>
+  <si>
+    <t>中文 (香港)</t>
+  </si>
+  <si>
+    <t>日本語</t>
+  </si>
+  <si>
+    <t>한국어</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color indexed="8"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -491,83 +653,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -867,884 +970,765 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="36.33203125"/>
-    <col min="2" max="2" customWidth="true" style="1" width="104.5546875"/>
-    <col min="3" max="3" width="40.0" customWidth="true"/>
-    <col min="4" max="4" width="40.0" customWidth="true"/>
+    <col min="1" max="1" width="36.33203125" customWidth="1"/>
+    <col min="2" max="2" width="104.5546875" style="1" customWidth="1"/>
+    <col min="3" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="0">
-        <is>
-          <t>Applied Language</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Data</t>
-        </is>
-      </c>
-      <c r="C1" t="s" s="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" t="s" s="1">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" ht="28.8" customHeight="1">
-      <c r="A2" t="inlineStr" s="0">
-        <is>
-          <t>Afrikaans</t>
-        </is>
-      </c>
-      <c r="B2" t="s" s="1">
+      <c r="D2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s" s="1">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s" s="1">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="28.8" customHeight="1">
-      <c r="A3" t="inlineStr" s="0">
-        <is>
-          <t>Azərbaycan</t>
-        </is>
-      </c>
-      <c r="B3" t="s" s="1">
+    <row r="4" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s" s="1">
+      <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s" s="1">
+      <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" ht="28.8" customHeight="1">
-      <c r="A4" t="inlineStr" s="0">
-        <is>
-          <t>Bahasa Indonesia</t>
-        </is>
-      </c>
-      <c r="B4" t="s" s="1">
+    <row r="5" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s" s="1">
+      <c r="C5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s" s="1">
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" ht="28.8" customHeight="1">
-      <c r="A5" t="inlineStr" s="0">
-        <is>
-          <t>Bosanski</t>
-        </is>
-      </c>
-      <c r="B5" t="s" s="1">
+    <row r="6" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s" s="1">
+      <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D5" t="s" s="1">
+      <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" ht="28.8" customHeight="1">
-      <c r="A6" t="inlineStr" s="0">
-        <is>
-          <t>Català</t>
-        </is>
-      </c>
-      <c r="B6" t="s" s="1">
+    <row r="7" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s" s="1">
+      <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D6" t="s" s="1">
+      <c r="D7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" ht="28.8" customHeight="1">
-      <c r="A7" t="inlineStr" s="0">
-        <is>
-          <t>Dansk</t>
-        </is>
-      </c>
-      <c r="B7" t="s" s="1">
+    <row r="8" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" t="s" s="1">
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D7" t="s" s="1">
+    </row>
+    <row r="9" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" ht="28.8" customHeight="1">
-      <c r="A8" t="inlineStr" s="0">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="B8" t="s" s="1">
+      <c r="C9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s" s="1">
+      <c r="D9" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" ht="28.8" customHeight="1">
-      <c r="A9" t="inlineStr" s="0">
-        <is>
-          <t>Eesti</t>
-        </is>
-      </c>
-      <c r="B9" t="s" s="1">
+    <row r="10" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s" s="1">
+      <c r="C10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s" s="1">
+    </row>
+    <row r="11" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" ht="28.8" customHeight="1">
-      <c r="A10" t="inlineStr" s="0">
-        <is>
-          <t>English (India)</t>
-        </is>
-      </c>
-      <c r="B10" t="s" s="1">
+      <c r="C13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D10" t="s" s="1">
+      <c r="D13" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" ht="28.8" customHeight="1">
-      <c r="A11" t="inlineStr" s="0">
-        <is>
-          <t>English (UK)</t>
-        </is>
-      </c>
-      <c r="B11" t="s" s="1">
-        <v>26</v>
-      </c>
-      <c r="C11" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D11" t="s" s="1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" ht="28.8" customHeight="1">
-      <c r="A12" t="inlineStr" s="0">
-        <is>
-          <t>English (US)</t>
-        </is>
-      </c>
-      <c r="B12" t="s" s="1">
-        <v>26</v>
-      </c>
-      <c r="C12" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D12" t="s" s="1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" ht="28.8" customHeight="1">
-      <c r="A13" t="inlineStr" s="0">
-        <is>
-          <t>Español (España)</t>
-        </is>
-      </c>
-      <c r="B13" t="s" s="1">
+    <row r="14" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C13" t="s" s="1">
+      <c r="C14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D13" t="s" s="1">
+      <c r="D14" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" ht="28.8" customHeight="1">
-      <c r="A14" t="inlineStr" s="0">
-        <is>
-          <t>Español (Latinoamérica)</t>
-        </is>
-      </c>
-      <c r="B14" t="s" s="1">
+    <row r="15" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C14" t="s" s="1">
+      <c r="C16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D14" t="s" s="1">
+      <c r="D16" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" ht="28.8" customHeight="1">
-      <c r="A15" t="inlineStr" s="0">
-        <is>
-          <t>Español (US)</t>
-        </is>
-      </c>
-      <c r="B15" t="s" s="1">
-        <v>31</v>
-      </c>
-      <c r="C15" t="s" s="1">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s" s="1">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" ht="28.8" customHeight="1">
-      <c r="A16" t="inlineStr" s="0">
-        <is>
-          <t>Euskara</t>
-        </is>
-      </c>
-      <c r="B16" t="s" s="1">
+    <row r="17" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C16" t="s" s="1">
+      <c r="C17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D16" t="s" s="1">
+      <c r="D17" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" ht="28.8" customHeight="1">
-      <c r="A17" t="inlineStr" s="0">
-        <is>
-          <t>Français</t>
-        </is>
-      </c>
-      <c r="B17" t="s" s="1">
+    <row r="18" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C17" t="s" s="1">
+      <c r="C18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D17" t="s" s="1">
+      <c r="D18" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" ht="28.8" customHeight="1">
-      <c r="A18" t="inlineStr" s="0">
-        <is>
-          <t>Français (Canada)</t>
-        </is>
-      </c>
-      <c r="B18" t="s" s="1">
+    <row r="19" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>163</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C18" t="s" s="1">
+      <c r="C19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D18" t="s" s="1">
+      <c r="D19" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>164</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" ht="28.8" customHeight="1">
-      <c r="A19" t="inlineStr" s="0">
-        <is>
-          <t>Hrvatski</t>
-        </is>
-      </c>
-      <c r="B19" t="s" s="1">
+      <c r="C20" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C19" t="s" s="1">
+      <c r="D20" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D19" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" ht="28.8" customHeight="1">
-      <c r="A20" t="inlineStr" s="0">
-        <is>
-          <t>Íslenska</t>
-        </is>
-      </c>
-      <c r="B20" t="s" s="1">
+    </row>
+    <row r="21" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>165</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C20" t="s" s="1">
+      <c r="C21" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D20" t="s" s="1">
+    </row>
+    <row r="22" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>166</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" ht="28.8" customHeight="1">
-      <c r="A21" t="inlineStr" s="0">
-        <is>
-          <t>Italiano</t>
-        </is>
-      </c>
-      <c r="B21" t="s" s="1">
+      <c r="C22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C21" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D21" t="s" s="1">
+      <c r="D22" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="22" ht="28.8" customHeight="1">
-      <c r="A22" t="inlineStr" s="0">
-        <is>
-          <t>Latviešu valoda</t>
-        </is>
-      </c>
-      <c r="B22" t="s" s="1">
+    <row r="23" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C22" t="s" s="1">
+      <c r="C23" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D22" t="s" s="1">
+      <c r="D23" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="23" ht="28.8" customHeight="1">
-      <c r="A23" t="inlineStr" s="0">
-        <is>
-          <t>Lietuvių</t>
-        </is>
-      </c>
-      <c r="B23" t="s" s="1">
+    <row r="24" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C23" t="s" s="1">
+      <c r="C24" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D23" t="s" s="1">
+      <c r="D24" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="24" ht="28.8" customHeight="1">
-      <c r="A24" t="inlineStr" s="0">
-        <is>
-          <t>Magyar</t>
-        </is>
-      </c>
-      <c r="B24" t="s" s="1">
+    <row r="25" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>169</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C24" t="s" s="1">
+      <c r="C25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D24" t="s" s="1">
+    </row>
+    <row r="26" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>170</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="25" ht="28.8" customHeight="1">
-      <c r="A25" t="inlineStr" s="0">
-        <is>
-          <t>Nederlands</t>
-        </is>
-      </c>
-      <c r="B25" t="s" s="1">
+      <c r="C26" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C25" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D25" t="s" s="1">
+      <c r="D26" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="26" ht="28.8" customHeight="1">
-      <c r="A26" t="inlineStr" s="0">
-        <is>
-          <t>Polski</t>
-        </is>
-      </c>
-      <c r="B26" t="s" s="1">
+    <row r="27" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C26" t="s" s="1">
+      <c r="C27" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D26" t="s" s="1">
+      <c r="D27" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="27" ht="28.8" customHeight="1">
-      <c r="A27" t="inlineStr" s="0">
-        <is>
-          <t>Português</t>
-        </is>
-      </c>
-      <c r="B27" t="s" s="1">
+    <row r="28" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>172</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C27" t="s" s="1">
+      <c r="C28" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D27" t="s" s="1">
+      <c r="D28" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="28" ht="28.8" customHeight="1">
-      <c r="A28" t="inlineStr" s="0">
-        <is>
-          <t>Português (Brasil)</t>
-        </is>
-      </c>
-      <c r="B28" t="s" s="1">
+    <row r="29" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>173</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s" s="1">
+      <c r="C29" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D28" t="s" s="1">
+      <c r="D29" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="29" ht="28.8" customHeight="1">
-      <c r="A29" t="inlineStr" s="0">
-        <is>
-          <t>Shqip</t>
-        </is>
-      </c>
-      <c r="B29" t="s" s="1">
+    <row r="30" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>174</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C29" t="s" s="1">
+      <c r="C30" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D29" t="s" s="1">
+      <c r="D30" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" ht="28.8" customHeight="1">
-      <c r="A30" t="inlineStr" s="0">
-        <is>
-          <t>Slovenščina</t>
-        </is>
-      </c>
-      <c r="B30" t="s" s="1">
+    <row r="31" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>175</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C30" t="s" s="1">
+      <c r="C31" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D30" t="s" s="1">
+      <c r="D31" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" ht="28.8" customHeight="1">
-      <c r="A31" t="inlineStr" s="0">
-        <is>
-          <t>Suomi</t>
-        </is>
-      </c>
-      <c r="B31" t="s" s="1">
+    <row r="32" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>176</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C31" t="s" s="1">
+      <c r="C32" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D31" t="s" s="1">
+      <c r="D32" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="32" ht="28.8" customHeight="1">
-      <c r="A32" t="inlineStr" s="0">
-        <is>
-          <t>Svenska</t>
-        </is>
-      </c>
-      <c r="B32" t="s" s="1">
+    <row r="33" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>177</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C32" t="s" s="1">
+      <c r="C33" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D32" t="s" s="1">
+      <c r="D33" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="33" ht="28.8" customHeight="1">
-      <c r="A33" t="inlineStr" s="0">
-        <is>
-          <t>Tiếng Việt</t>
-        </is>
-      </c>
-      <c r="B33" t="s" s="1">
+    <row r="34" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>178</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C33" t="s" s="1">
+      <c r="C34" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D33" t="s" s="1">
+      <c r="D34" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="34" ht="28.8" customHeight="1">
-      <c r="A34" t="inlineStr" s="0">
-        <is>
-          <t>Türkçe</t>
-        </is>
-      </c>
-      <c r="B34" t="s" s="1">
+    <row r="35" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>179</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C34" t="s" s="1">
+      <c r="C35" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D34" t="s" s="1">
+      <c r="D35" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="35" ht="28.8" customHeight="1">
-      <c r="A35" t="inlineStr" s="0">
-        <is>
-          <t>Беларуская</t>
-        </is>
-      </c>
-      <c r="B35" t="s" s="1">
+    <row r="36" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>180</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C35" t="s" s="1">
+      <c r="C36" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D35" t="s" s="1">
+      <c r="D36" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="36" ht="28.8" customHeight="1">
-      <c r="A36" t="inlineStr" s="0">
-        <is>
-          <t>Български</t>
-        </is>
-      </c>
-      <c r="B36" t="s" s="1">
+    <row r="37" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C36" t="s" s="1">
+      <c r="C37" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D36" t="s" s="1">
+      <c r="D37" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="37" ht="28.8" customHeight="1">
-      <c r="A37" t="inlineStr" s="0">
-        <is>
-          <t>Русский</t>
-        </is>
-      </c>
-      <c r="B37" t="s" s="1">
+    <row r="38" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>182</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C37" t="s" s="1">
+      <c r="C38" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D37" t="s" s="1">
+      <c r="D38" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="38" ht="28.8" customHeight="1">
-      <c r="A38" t="inlineStr" s="0">
-        <is>
-          <t>Українська</t>
-        </is>
-      </c>
-      <c r="B38" t="s" s="1">
+    <row r="39" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>183</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C38" t="s" s="1">
+      <c r="C39" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D38" t="s" s="1">
+    </row>
+    <row r="40" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>184</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="39" ht="28.8" customHeight="1">
-      <c r="A39" t="inlineStr" s="0">
-        <is>
-          <t>Ελληνικά</t>
-        </is>
-      </c>
-      <c r="B39" t="s" s="1">
+      <c r="C40" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C39" t="s" s="1">
-        <v>19</v>
-      </c>
-      <c r="D39" t="s" s="1">
+      <c r="D40" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="40" ht="28.8" customHeight="1">
-      <c r="A40" t="inlineStr" s="0">
-        <is>
-          <t>Հայերեն</t>
-        </is>
-      </c>
-      <c r="B40" t="s" s="1">
+    <row r="41" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>185</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C40" t="s" s="1">
+      <c r="C41" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D40" t="s" s="1">
+      <c r="D41" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="41" ht="28.8" customHeight="1">
-      <c r="A41" t="inlineStr" s="0">
-        <is>
-          <t>עברית</t>
-        </is>
-      </c>
-      <c r="B41" t="s" s="1">
+    <row r="42" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>186</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C41" t="s" s="1">
+      <c r="C42" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D41" t="s" s="1">
+      <c r="D42" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="42" ht="28.8" customHeight="1">
-      <c r="A42" t="inlineStr" s="0">
-        <is>
-          <t>العربية</t>
-        </is>
-      </c>
-      <c r="B42" t="s" s="1">
+    <row r="43" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>187</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C42" t="s" s="1">
+      <c r="C43" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D42" t="s" s="1">
+      <c r="D43" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="43" ht="28.8" customHeight="1">
-      <c r="A43" t="inlineStr" s="0">
-        <is>
-          <t>فارسی</t>
-        </is>
-      </c>
-      <c r="B43" t="s" s="1">
+    <row r="44" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>188</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C43" t="s" s="1">
+      <c r="C44" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D43" t="s" s="1">
+      <c r="D44" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="44" ht="28.8" customHeight="1">
-      <c r="A44" t="inlineStr" s="0">
-        <is>
-          <t>हिन्दी</t>
-        </is>
-      </c>
-      <c r="B44" t="s" s="1">
+    <row r="45" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>189</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C44" t="s" s="1">
+      <c r="C45" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D44" t="s" s="1">
+      <c r="D45" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="45" ht="28.8" customHeight="1">
-      <c r="A45" t="inlineStr" s="0">
-        <is>
-          <t>বাংলা</t>
-        </is>
-      </c>
-      <c r="B45" t="s" s="1">
+    <row r="46" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>190</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C45" t="s" s="1">
+      <c r="C46" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D45" t="s" s="1">
+      <c r="D46" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="46" ht="28.8" customHeight="1">
-      <c r="A46" t="inlineStr" s="0">
-        <is>
-          <t>ਪੰਜਾਬੀ</t>
-        </is>
-      </c>
-      <c r="B46" t="s" s="1">
+    <row r="47" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>191</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C46" t="s" s="1">
+      <c r="C47" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D46" t="s" s="1">
+      <c r="D47" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="47" ht="28.8" customHeight="1">
-      <c r="A47" t="inlineStr" s="0">
-        <is>
-          <t>ગુજરાતી</t>
-        </is>
-      </c>
-      <c r="B47" t="s" s="1">
+    <row r="48" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>192</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C47" t="s" s="1">
+      <c r="C48" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D47" t="s" s="1">
+      <c r="D48" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="48" ht="28.8" customHeight="1">
-      <c r="A48" t="inlineStr" s="0">
-        <is>
-          <t>தமிழ்</t>
-        </is>
-      </c>
-      <c r="B48" t="s" s="1">
+    <row r="49" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C48" t="s" s="1">
+      <c r="C49" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D48" t="s" s="1">
+      <c r="D49" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="49" ht="28.8" customHeight="1">
-      <c r="A49" t="inlineStr" s="0">
-        <is>
-          <t>తెలుగు</t>
-        </is>
-      </c>
-      <c r="B49" t="s" s="1">
+    <row r="50" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>194</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C49" t="s" s="1">
+      <c r="C50" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D49" t="s" s="1">
+      <c r="D50" s="1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="50" ht="28.8" customHeight="1">
-      <c r="A50" t="inlineStr" s="0">
-        <is>
-          <t>中文 (简体)</t>
-        </is>
-      </c>
-      <c r="B50" t="s" s="1">
+    <row r="51" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>195</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C50" t="s" s="1">
+      <c r="C51" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D50" t="s" s="1">
+      <c r="D51" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="51" ht="28.8" customHeight="1">
-      <c r="A51" t="inlineStr" s="0">
-        <is>
-          <t>中文 (繁體)</t>
-        </is>
-      </c>
-      <c r="B51" t="s" s="1">
+    <row r="52" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>196</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C51" t="s" s="1">
+      <c r="C52" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D51" t="s" s="1">
+      <c r="D52" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="52" ht="28.8" customHeight="1">
-      <c r="A52" t="inlineStr" s="0">
-        <is>
-          <t>中文 (香港)</t>
-        </is>
-      </c>
-      <c r="B52" t="s" s="1">
+    <row r="53" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>197</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C52" t="s" s="1">
+      <c r="C53" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D52" t="s" s="1">
+      <c r="D53" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="53" ht="28.8" customHeight="1">
-      <c r="A53" t="inlineStr" s="0">
-        <is>
-          <t>日本語</t>
-        </is>
-      </c>
-      <c r="B53" t="s" s="1">
+    <row r="54" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>198</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C53" t="s" s="1">
+      <c r="C54" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D53" t="s" s="1">
+      <c r="D54" s="1" t="s">
         <v>143</v>
-      </c>
-    </row>
-    <row r="54" ht="28.8" customHeight="1">
-      <c r="A54" t="inlineStr" s="0">
-        <is>
-          <t>한국어</t>
-        </is>
-      </c>
-      <c r="B54" t="s" s="1">
-        <v>144</v>
-      </c>
-      <c r="C54" t="s" s="1">
-        <v>145</v>
-      </c>
-      <c r="D54" t="s" s="1">
-        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding the good data back
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/verifyingSideMenuLanguageAsInSettings.xlsx
@@ -908,7 +908,9 @@
       <c r="B2" t="s" s="1">
         <v>3</v>
       </c>
-      <c r="C2" s="1"/>
+      <c r="C2" t="s" s="1">
+        <v>4</v>
+      </c>
       <c r="D2" t="s" s="1">
         <v>5</v>
       </c>

</xml_diff>